<commit_message>
﻿Fix Arabic test titles, language switcher pattern and overflow check
- Test titles use the stable section ID instead of the section name, which contains characters the Playwright worker lookup rejects (8 Arabic tests were not found).
- Arabic language-switcher pattern accepts the live label EN; the English test now uses the same pattern.
- Horizontal-overflow check counts only elements that extend past the viewport without a clipping ancestor, so carousel slides inside overflow-hidden containers no longer fail.
- CSV report takes the feature name from the test plan.

Arabic run: 47 passed, 5 failed (was 34 passed, 18 failed).

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/ar/run-report-2026-10-12.xlsx
+++ b/state/ar/run-report-2026-10-12.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="276">
   <si>
     <t>Metric</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Pass rate (PASS / total)</t>
   </si>
   <si>
-    <t>65.4%</t>
+    <t>90.4%</t>
   </si>
   <si>
     <t>Results by device</t>
@@ -68,7 +68,7 @@
     <t>chromium</t>
   </si>
   <si>
-    <t>PASS 34 | FAIL 18 | FLAKY 0 | NOT RUN 0</t>
+    <t>PASS 47 | FAIL 5 | FLAKY 0 | NOT RUN 0</t>
   </si>
   <si>
     <t>Test case ID</t>
@@ -110,7 +110,7 @@
     <t>TC-HOME-AR-002</t>
   </si>
   <si>
-    <t>homepage-buttons.spec.js</t>
+    <t>تسوّّق حسب الماركة — buttons</t>
   </si>
   <si>
     <t>TC-HOME-AR-002: تسوّّق حسب الماركة — buttons behave as expected</t>
@@ -119,106 +119,139 @@
     <t>matches expected</t>
   </si>
   <si>
-    <t>9068</t>
+    <t>5787</t>
   </si>
   <si>
     <t>TC-HOME-AR-007</t>
   </si>
   <si>
-    <t>TC-HOME-AR-007: تابلتك الجديد مع كل اللي تحتاجه. — buttons behave as expected</t>
-  </si>
-  <si>
-    <t>1893</t>
+    <t>تابلتك الجديد مع كل اللي تحتاجه. — buttons</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-007: ارتق إلى آيفون 18 — buttons behave as expected</t>
+  </si>
+  <si>
+    <t>1681</t>
   </si>
   <si>
     <t>TC-HOME-AR-011</t>
   </si>
   <si>
-    <t>TC-HOME-AR-011: اشتر 1 واحصل على 1 مجانا — buttons behave as expected</t>
-  </si>
-  <si>
-    <t>1788</t>
+    <t>اشتر 1 واحصل على 1 مجانا — buttons</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-011: جوالك الجديد وكل اللي تحتاجه معه. — buttons behave as expected</t>
+  </si>
+  <si>
+    <t>1317</t>
   </si>
   <si>
     <t>TC-HOME-AR-015</t>
   </si>
   <si>
-    <t>TC-HOME-AR-015: PS5 تسوق باقات — buttons behave as expected</t>
-  </si>
-  <si>
-    <t>1695</t>
+    <t>PS5 تسوق باقات — buttons</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-015: اختاروا عطراً يستحق أن يكون هدية. — buttons behave as expected</t>
+  </si>
+  <si>
+    <t>1213</t>
   </si>
   <si>
     <t>TC-HOME-AR-019</t>
   </si>
   <si>
-    <t>TC-HOME-AR-019: اختاروا عطراً يستحق أن يكون هدية. — buttons behave as expected</t>
-  </si>
-  <si>
-    <t>1662</t>
+    <t>اختاروا عطراً يستحق أن يكون هدية. — buttons</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-019: سماعات ألعاب — buttons behave as expected</t>
+  </si>
+  <si>
+    <t>1485</t>
   </si>
   <si>
     <t>TC-HOME-AR-023</t>
   </si>
   <si>
+    <t>عروض الأسبوع — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-023: عروض الأسبوع — buttons behave as expected</t>
   </si>
   <si>
-    <t>1856</t>
+    <t>1311</t>
   </si>
   <si>
     <t>TC-HOME-AR-027</t>
   </si>
   <si>
+    <t>المنتجات الأكثر شعبية — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-027: المنتجات الأكثر شعبية — buttons behave as expected</t>
   </si>
   <si>
-    <t>2861</t>
+    <t>2184</t>
   </si>
   <si>
     <t>TC-HOME-AR-033</t>
   </si>
   <si>
+    <t>جديد في مجموعتنا — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-033: جديد في مجموعتنا — buttons behave as expected</t>
   </si>
   <si>
-    <t>2663</t>
+    <t>1603</t>
   </si>
   <si>
     <t>TC-HOME-AR-039</t>
   </si>
   <si>
+    <t>منتجات على ذوقك — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-039: منتجات على ذوقك — buttons behave as expected</t>
   </si>
   <si>
-    <t>2211</t>
+    <t>1781</t>
   </si>
   <si>
     <t>TC-HOME-AR-043</t>
   </si>
   <si>
+    <t>منتجات مناسبة لكل عمر — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-043: منتجات مناسبة لكل عمر — buttons behave as expected</t>
   </si>
   <si>
-    <t>2201</t>
+    <t>1380</t>
   </si>
   <si>
     <t>TC-HOME-AR-046</t>
   </si>
   <si>
+    <t>نصنع السعادة , نخلق الذكريات — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-046: نصنع السعادة , نخلق الذكريات — buttons behave as expected</t>
   </si>
   <si>
-    <t>2807</t>
+    <t>1650</t>
   </si>
   <si>
     <t>TC-HOME-AR-050</t>
   </si>
   <si>
+    <t>تسوق حسب الفئة — buttons</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-050: تسوق حسب الفئة — buttons behave as expected</t>
   </si>
   <si>
-    <t>3850</t>
+    <t>3108</t>
   </si>
   <si>
     <t>discover and map the homepage</t>
@@ -227,352 +260,424 @@
     <t>Homepage discovery</t>
   </si>
   <si>
-    <t>19592</t>
+    <t>16717</t>
   </si>
   <si>
     <t>TC-HOME-AR-001</t>
   </si>
   <si>
-    <t>homepage-links.spec.js</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-001: تسوّّق حسب الماركة — every link resolves</t>
+    <t>تسوّّق حسب الماركة — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-001: HOME-SEC-AR-001 — every link resolves</t>
+  </si>
+  <si>
+    <t>11648</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-006</t>
+  </si>
+  <si>
+    <t>تابلتك الجديد مع كل اللي تحتاجه. — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-006: HOME-SEC-AR-002 — every link resolves</t>
+  </si>
+  <si>
+    <t>1816</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-010</t>
+  </si>
+  <si>
+    <t>اشتر 1 واحصل على 1 مجانا — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-010: HOME-SEC-AR-003 — every link resolves</t>
+  </si>
+  <si>
+    <t>1486</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-014</t>
+  </si>
+  <si>
+    <t>PS5 تسوق باقات — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-014: HOME-SEC-AR-004 — every link resolves</t>
+  </si>
+  <si>
+    <t>1459</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-018</t>
+  </si>
+  <si>
+    <t>اختاروا عطراً يستحق أن يكون هدية. — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-018: HOME-SEC-AR-005 — every link resolves</t>
+  </si>
+  <si>
+    <t>1423</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-022</t>
+  </si>
+  <si>
+    <t>عروض الأسبوع — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-022: HOME-SEC-AR-006 — every link resolves</t>
+  </si>
+  <si>
+    <t>1160</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-026</t>
+  </si>
+  <si>
+    <t>المنتجات الأكثر شعبية — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-026: HOME-SEC-AR-007 — every link resolves</t>
+  </si>
+  <si>
+    <t>1850</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-030</t>
+  </si>
+  <si>
+    <t>استكشف جواهرنا الخفية — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-030: HOME-SEC-AR-008 — every link resolves</t>
+  </si>
+  <si>
+    <t>571</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-032</t>
+  </si>
+  <si>
+    <t>جديد في مجموعتنا — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-032: HOME-SEC-AR-009 — every link resolves</t>
+  </si>
+  <si>
+    <t>2709</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-036</t>
+  </si>
+  <si>
+    <t>عروض اس تثنائية💖 — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-036: HOME-SEC-AR-010 — every link resolves</t>
+  </si>
+  <si>
+    <t>1240</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-038</t>
+  </si>
+  <si>
+    <t>منتجات على ذوقك — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-038: HOME-SEC-AR-011 — every link resolves</t>
+  </si>
+  <si>
+    <t>6577</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-042</t>
+  </si>
+  <si>
+    <t>منتجات مناسبة لكل عمر — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-042: HOME-SEC-AR-012 — every link resolves</t>
+  </si>
+  <si>
+    <t>2163</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-048</t>
+  </si>
+  <si>
+    <t>⭐ بتقييم 4.7 على قوقل — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-048: HOME-SEC-AR-014 — every link resolves</t>
+  </si>
+  <si>
+    <t>2217</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-049</t>
+  </si>
+  <si>
+    <t>تسوق حسب الفئة — links</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-049: HOME-SEC-AR-019 — every link resolves</t>
   </si>
   <si>
     <t>[31mTest timeout of 60000ms exceeded.[39m</t>
   </si>
   <si>
-    <t>65298</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--d2258-ماركة-—-every-link-resolves-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--d2258-ماركة-—-every-link-resolves-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--d2258-ماركة-—-every-link-resolves-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--d2258-ماركة-—-every-link-resolves-chromium\trace.zip</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-006</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-006: تابلتك الجديد مع كل اللي تحتاجه. — every link resolves</t>
-  </si>
-  <si>
-    <t>Test not found in the worker process. Make sure test title does not change.</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-010</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-010: اشتر 1 واحصل على 1 مجانا — every link resolves</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-014</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-014: PS5 تسوق باقات — every link resolves</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-018</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-018: اختاروا عطراً يستحق أن يكون هدية. — every link resolves</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-022</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-022: عروض الأسبوع — every link resolves</t>
-  </si>
-  <si>
-    <t>10132</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-026</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-026: المنتجات الأكثر شعبية — every link resolves</t>
-  </si>
-  <si>
-    <t>5289</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-030</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-030: استكشف جواهرنا الخفية — every link resolves</t>
-  </si>
-  <si>
-    <t>2784</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-032</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-032: جديد في مجموعتنا — every link resolves</t>
-  </si>
-  <si>
-    <t>21400</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-036</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-036: عروض اس تثنائية💖 — every link resolves</t>
-  </si>
-  <si>
-    <t>16714</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-038</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-038: منتجات على ذوقك — every link resolves</t>
-  </si>
-  <si>
-    <t>26613</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-042</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-042: منتجات مناسبة لكل عمر — every link resolves</t>
-  </si>
-  <si>
-    <t>27747</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-048</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-048: ⭐ بتقييم 4.7 على قوقل — every link resolves</t>
-  </si>
-  <si>
-    <t>1887</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-049</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-049: تسوق حسب الفئة — every link resolves</t>
-  </si>
-  <si>
-    <t>66039</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--f382f-الفئة-—-every-link-resolves-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--f382f-الفئة-—-every-link-resolves-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--f382f-الفئة-—-every-link-resolves-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--f382f-الفئة-—-every-link-resolves-chromium\trace.zip</t>
+    <t>64935</t>
+  </si>
+  <si>
+    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--9d7ee-R-019-—-every-link-resolves-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--9d7ee-R-019-—-every-link-resolves-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--9d7ee-R-019-—-every-link-resolves-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-links-TC-HOME-AR--9d7ee-R-019-—-every-link-resolves-chromium\trace.zip</t>
   </si>
   <si>
     <t>TC-HOME-AR-064</t>
   </si>
   <si>
-    <t>homepage-negative.spec.js</t>
+    <t>Negative &amp; edge — interaction robustness</t>
   </si>
   <si>
     <t>TC-HOME-AR-064: Global negative/edge — interaction robustness</t>
   </si>
   <si>
-    <t>11599</t>
+    <t>Error: No Add to Cart button found for rapid-click check</t>
+  </si>
+  <si>
+    <t>Error: No Add to Cart button found for rapid-click check Clicking a product card did not navigate away from the homepage (still at https://thekanaa.com/ar-sa/) Back navigation did not return to homepage (at about:blank) — reproduced once; rerun to confirm before filing as a bug [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m [32m- Expected - 1[39m [31m+ Received + 5[39m [32m- Array [][39m [31m+ Array [[39m [31m+ "No Add to Cart</t>
+  </si>
+  <si>
+    <t>11632</t>
+  </si>
+  <si>
+    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-negative-TC-HOME--f0b30-ge-—-interaction-robustness-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-negative-TC-HOME--f0b30-ge-—-interaction-robustness-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-negative-TC-HOME--f0b30-ge-—-interaction-robustness-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-negative-TC-HOME--f0b30-ge-—-interaction-robustness-chromium\trace.zip</t>
   </si>
   <si>
     <t>TC-HOME-AR-067</t>
   </si>
   <si>
+    <t>Performance observation — initial load</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-067: Global performance observation — initial load</t>
   </si>
   <si>
-    <t>2466</t>
+    <t>4456</t>
   </si>
   <si>
     <t>TC-HOME-AR-008</t>
   </si>
   <si>
-    <t>homepage-products.spec.js</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-008: تابلتك الجديد مع كل اللي تحتاجه. — sampled product cards</t>
+    <t>تابلتك الجديد مع كل اللي تحتاجه. — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-008: HOME-SEC-AR-002 — sampled product cards</t>
+  </si>
+  <si>
+    <t>Error: smoke Add to Cart (sample #0) failed: locator.click: Timeout 5000ms exceeded.</t>
+  </si>
+  <si>
+    <t>Error: smoke Add to Cart (sample #0) failed: locator.click: Timeout 5000ms exceeded. Call log: [2m - waiting for getByRole('button', { name: /إضافة إلى السلة/ }).first()[22m [2m - locator — see README "Known site quirks" re: throttling before filing as a bug [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m [32m- Expected - 1[39m [31m+ Received + 6[39m [32m- Array [][39m [31m+ Array [[39m [31m+ "smoke Add to Cart (sample #0) f</t>
+  </si>
+  <si>
+    <t>32661</t>
+  </si>
+  <si>
+    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-products-TC-HOME--1e8aa-002-—-sampled-product-cards-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-products-TC-HOME--1e8aa-002-—-sampled-product-cards-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-products-TC-HOME--1e8aa-002-—-sampled-product-cards-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-products-TC-HOME--1e8aa-002-—-sampled-product-cards-chromium\trace.zip</t>
   </si>
   <si>
     <t>TC-HOME-AR-012</t>
   </si>
   <si>
-    <t>TC-HOME-AR-012: اشتر 1 واحصل على 1 مجانا — sampled product cards</t>
+    <t>اشتر 1 واحصل على 1 مجانا — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-012: HOME-SEC-AR-003 — sampled product cards</t>
+  </si>
+  <si>
+    <t>22990</t>
   </si>
   <si>
     <t>TC-HOME-AR-016</t>
   </si>
   <si>
-    <t>TC-HOME-AR-016: PS5 تسوق باقات — sampled product cards</t>
+    <t>PS5 تسوق باقات — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-016: HOME-SEC-AR-004 — sampled product cards</t>
+  </si>
+  <si>
+    <t>24257</t>
   </si>
   <si>
     <t>TC-HOME-AR-020</t>
   </si>
   <si>
-    <t>TC-HOME-AR-020: اختاروا عطراً يستحق أن يكون هدية. — sampled product cards</t>
+    <t>اختاروا عطراً يستحق أن يكون هدية. — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-020: HOME-SEC-AR-005 — sampled product cards</t>
+  </si>
+  <si>
+    <t>22596</t>
   </si>
   <si>
     <t>TC-HOME-AR-024</t>
   </si>
   <si>
-    <t>TC-HOME-AR-024: عروض الأسبوع — sampled product cards</t>
-  </si>
-  <si>
-    <t>22129</t>
+    <t>عروض الأسبوع — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-024: HOME-SEC-AR-006 — sampled product cards</t>
+  </si>
+  <si>
+    <t>20031</t>
   </si>
   <si>
     <t>TC-HOME-AR-028</t>
   </si>
   <si>
-    <t>TC-HOME-AR-028: المنتجات الأكثر شعبية — sampled product cards</t>
-  </si>
-  <si>
-    <t>21478</t>
+    <t>المنتجات الأكثر شعبية — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-028: HOME-SEC-AR-007 — sampled product cards</t>
+  </si>
+  <si>
+    <t>23599</t>
   </si>
   <si>
     <t>TC-HOME-AR-034</t>
   </si>
   <si>
-    <t>TC-HOME-AR-034: جديد في مجموعتنا — sampled product cards</t>
-  </si>
-  <si>
-    <t>22286</t>
+    <t>جديد في مجموعتنا — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-034: HOME-SEC-AR-009 — sampled product cards</t>
+  </si>
+  <si>
+    <t>24550</t>
   </si>
   <si>
     <t>TC-HOME-AR-040</t>
   </si>
   <si>
-    <t>TC-HOME-AR-040: منتجات على ذوقك — sampled product cards</t>
-  </si>
-  <si>
-    <t>18227</t>
+    <t>منتجات على ذوقك — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-040: HOME-SEC-AR-011 — sampled product cards</t>
+  </si>
+  <si>
+    <t>19779</t>
   </si>
   <si>
     <t>TC-HOME-AR-044</t>
   </si>
   <si>
-    <t>TC-HOME-AR-044: منتجات مناسبة لكل عمر — sampled product cards</t>
-  </si>
-  <si>
-    <t>21530</t>
+    <t>منتجات مناسبة لكل عمر — product cards</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-044: HOME-SEC-AR-012 — sampled product cards</t>
+  </si>
+  <si>
+    <t>21403</t>
   </si>
   <si>
     <t>TC-HOME-AR-053</t>
   </si>
   <si>
-    <t>homepage-responsive.spec.js</t>
+    <t>Responsive — Desktop 1440x900</t>
   </si>
   <si>
     <t>TC-HOME-AR-053: responsive at Desktop 1440x900</t>
   </si>
   <si>
-    <t>4851</t>
+    <t>4808</t>
   </si>
   <si>
     <t>TC-HOME-AR-054</t>
   </si>
   <si>
+    <t>Responsive — Desktop 1920x1080</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-054: responsive at Desktop 1920x1080</t>
   </si>
   <si>
-    <t>5097</t>
+    <t>6464</t>
   </si>
   <si>
     <t>TC-HOME-AR-055</t>
   </si>
   <si>
+    <t>Responsive — Tablet 1024x768</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-055: responsive at Tablet 1024x768</t>
   </si>
   <si>
-    <t>Error: Horizontal overflow at Tablet 1024x768</t>
-  </si>
-  <si>
-    <t>Error: Horizontal overflow at Tablet 1024x768 [2mexpect([22m[31mreceived[39m[2m).[22mtoBeLessThanOrEqual[2m([22m[32mexpected[39m[2m)[22m Expected: &lt;= [32m1026[39m Received: [31m1049[39m 61 | }); 62 | &gt; 63 | expect(overflow.scrollWidth, `Horizontal overflow at ${vp.name}`).toBeLessThanOrEqual(overflow.clientWidth + 2); | ^ 64 | }); 65 | } 66 | at C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\tests\homepage\homepage-responsive.spec.js:63:71</t>
-  </si>
-  <si>
-    <t>5922</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-585f7-sponsive-at-Tablet-1024x768-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-585f7-sponsive-at-Tablet-1024x768-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-585f7-sponsive-at-Tablet-1024x768-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-585f7-sponsive-at-Tablet-1024x768-chromium\trace.zip</t>
+    <t>4486</t>
   </si>
   <si>
     <t>TC-HOME-AR-056</t>
   </si>
   <si>
+    <t>Responsive — Tablet 768x1024</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-056: responsive at Tablet 768x1024</t>
   </si>
   <si>
-    <t>Error: Horizontal overflow at Tablet 768x1024</t>
-  </si>
-  <si>
-    <t>Error: Horizontal overflow at Tablet 768x1024 [2mexpect([22m[31mreceived[39m[2m).[22mtoBeLessThanOrEqual[2m([22m[32mexpected[39m[2m)[22m Expected: &lt;= [32m770[39m Received: [31m793[39m 61 | }); 62 | &gt; 63 | expect(overflow.scrollWidth, `Horizontal overflow at ${vp.name}`).toBeLessThanOrEqual(overflow.clientWidth + 2); | ^ 64 | }); 65 | } 66 | at C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\tests\homepage\homepage-responsive.spec.js:63:71</t>
-  </si>
-  <si>
-    <t>6131</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0e274-sponsive-at-Tablet-768x1024-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0e274-sponsive-at-Tablet-768x1024-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0e274-sponsive-at-Tablet-768x1024-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0e274-sponsive-at-Tablet-768x1024-chromium\trace.zip</t>
+    <t>5033</t>
   </si>
   <si>
     <t>TC-HOME-AR-057</t>
   </si>
   <si>
+    <t>Responsive — Mobile 390x844</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-057: responsive at Mobile 390x844</t>
   </si>
   <si>
-    <t>Error: Horizontal overflow at Mobile 390x844</t>
-  </si>
-  <si>
-    <t>Error: Horizontal overflow at Mobile 390x844 [2mexpect([22m[31mreceived[39m[2m).[22mtoBeLessThanOrEqual[2m([22m[32mexpected[39m[2m)[22m Expected: &lt;= [32m392[39m Received: [31m415[39m 61 | }); 62 | &gt; 63 | expect(overflow.scrollWidth, `Horizontal overflow at ${vp.name}`).toBeLessThanOrEqual(overflow.clientWidth + 2); | ^ 64 | }); 65 | } 66 | at C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\tests\homepage\homepage-responsive.spec.js:63:71</t>
-  </si>
-  <si>
-    <t>4757</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-f8b33-esponsive-at-Mobile-390x844-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-f8b33-esponsive-at-Mobile-390x844-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-f8b33-esponsive-at-Mobile-390x844-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-f8b33-esponsive-at-Mobile-390x844-chromium\trace.zip</t>
+    <t>3958</t>
   </si>
   <si>
     <t>TC-HOME-AR-058</t>
   </si>
   <si>
+    <t>Responsive — Mobile 393x852</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-058: responsive at Mobile 393x852</t>
   </si>
   <si>
-    <t>Error: Horizontal overflow at Mobile 393x852</t>
-  </si>
-  <si>
-    <t>Error: Horizontal overflow at Mobile 393x852 [2mexpect([22m[31mreceived[39m[2m).[22mtoBeLessThanOrEqual[2m([22m[32mexpected[39m[2m)[22m Expected: &lt;= [32m395[39m Received: [31m418[39m 61 | }); 62 | &gt; 63 | expect(overflow.scrollWidth, `Horizontal overflow at ${vp.name}`).toBeLessThanOrEqual(overflow.clientWidth + 2); | ^ 64 | }); 65 | } 66 | at C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\tests\homepage\homepage-responsive.spec.js:63:71</t>
-  </si>
-  <si>
-    <t>4573</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0ae07-esponsive-at-Mobile-393x852-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0ae07-esponsive-at-Mobile-393x852-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0ae07-esponsive-at-Mobile-393x852-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-0ae07-esponsive-at-Mobile-393x852-chromium\trace.zip</t>
+    <t>3715</t>
   </si>
   <si>
     <t>TC-HOME-AR-059</t>
   </si>
   <si>
+    <t>Responsive — Mobile 412x915</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-059: responsive at Mobile 412x915</t>
   </si>
   <si>
-    <t>Error: Horizontal overflow at Mobile 412x915</t>
-  </si>
-  <si>
-    <t>Error: Horizontal overflow at Mobile 412x915 [2mexpect([22m[31mreceived[39m[2m).[22mtoBeLessThanOrEqual[2m([22m[32mexpected[39m[2m)[22m Expected: &lt;= [32m414[39m Received: [31m437[39m 61 | }); 62 | &gt; 63 | expect(overflow.scrollWidth, `Horizontal overflow at ${vp.name}`).toBeLessThanOrEqual(overflow.clientWidth + 2); | ^ 64 | }); 65 | } 66 | at C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\tests\homepage\homepage-responsive.spec.js:63:71</t>
-  </si>
-  <si>
-    <t>5376</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-5b373-esponsive-at-Mobile-412x915-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-5b373-esponsive-at-Mobile-412x915-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-5b373-esponsive-at-Mobile-412x915-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-responsive-TC-HOM-5b373-esponsive-at-Mobile-412x915-chromium\trace.zip</t>
+    <t>5344</t>
   </si>
   <si>
     <t>TC-HOME-AR-003</t>
   </si>
   <si>
-    <t>homepage-sliders.spec.js</t>
-  </si>
-  <si>
-    <t>TC-HOME-AR-003: تسوّّق حسب الماركة — carousel navigation</t>
+    <t>تسوّّق حسب الماركة — carousel</t>
+  </si>
+  <si>
+    <t>TC-HOME-AR-003: HOME-SEC-AR-001 — carousel navigation</t>
   </si>
   <si>
     <t>TimeoutError: locator.click: Timeout 15000ms exceeded.</t>
@@ -581,10 +686,10 @@
     <t>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: [2m - waiting for getByRole('button', { name: /previous/i }).first()[22m [2m - locator resolved to &lt;button type="button" data-role="none" class="slick-arrow slick-prev"&gt; Previous&lt;/button&gt;[22m [2m - attempting click action[22m [2m 2 × waiting for element to be visible, enabled and stable[22m [2m - element is visible, enabled and stable[22m [2m - scrolling into view if needed[22m [2m - done scrolling[22m [2m - &lt;div dir</t>
   </si>
   <si>
-    <t>28781</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-12683-ماركة-—-carousel-navigation-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-12683-ماركة-—-carousel-navigation-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-12683-ماركة-—-carousel-navigation-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-12683-ماركة-—-carousel-navigation-chromium\trace.zip</t>
+    <t>30024</t>
+  </si>
+  <si>
+    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-ca077-R-001-—-carousel-navigation-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-ca077-R-001-—-carousel-navigation-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-ca077-R-001-—-carousel-navigation-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-sliders-TC-HOME-A-ca077-R-001-—-carousel-navigation-chromium\trace.zip</t>
   </si>
   <si>
     <t>HOME-IMG-SWEEP</t>
@@ -596,49 +701,49 @@
     <t>HOME-IMG-SWEEP: broken-image check across all sections</t>
   </si>
   <si>
-    <t>10295</t>
+    <t>10362</t>
   </si>
   <si>
     <t>TC-HOME-AR-063</t>
   </si>
   <si>
+    <t>Accessibility — keyboard &amp; names</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-063: Global accessibility — keyboard reachability &amp; accessible names</t>
   </si>
   <si>
-    <t>5795</t>
+    <t>4980</t>
   </si>
   <si>
     <t>TC-HOME-AR-066</t>
   </si>
   <si>
+    <t>Localization — switch to English</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-066: Global localization — switch to English</t>
   </si>
   <si>
-    <t>Error: Language switcher control not found by expected accessible name (pattern: /^EN$/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error: Language switcher control not found by expected accessible name (pattern: /^EN$/) [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m [32m- Expected - 1[39m [31m+ Received + 3[39m [32m- Array [][39m [31m+ Array [[39m [31m+ "Language switcher control not found by expected accessible name (pattern: /^EN$/)",[39m [31m+ ][39m 156 | actualResult: status === 'PASS' ? `Switched to ${targetLocaleLabel} cleanly with no overflow.` </t>
-  </si>
-  <si>
-    <t>3131</t>
-  </si>
-  <si>
-    <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-066-219e1-ization-—-switch-to-English-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-066-219e1-ization-—-switch-to-English-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-066-219e1-ization-—-switch-to-English-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-066-219e1-ization-—-switch-to-English-chromium\trace.zip</t>
+    <t>4515</t>
   </si>
   <si>
     <t>TC-HOME-AR-065</t>
   </si>
   <si>
+    <t>Console &amp; network health</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-065: Global console &amp; network health — first-party only</t>
   </si>
   <si>
-    <t>Error: POST https://thekanaa.com/ar-sa/ -&gt; net::ERR_ABORTED</t>
-  </si>
-  <si>
-    <t>Error: POST https://thekanaa.com/ar-sa/ -&gt; net::ERR_ABORTED GET https://thekanaa.com/ar-sa/gaming-consoles.html?_rsc=pm4ao -&gt; net::ERR_ABORTED GET https://thekanaa.com/ar-sa/mobile-phones-tablets.html?_rsc=pm4ao -&gt; net::ERR_ABORTED [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m [32m- Expected - 1[39m [31m+ Received + 5[39m [32m- Array [][39m [31m+ Array [[39m [31m+ "POST https://thekanaa.com/ar-sa/ -&gt; net::ERR_ABORTED",[39m </t>
-  </si>
-  <si>
-    <t>8885</t>
+    <t>Error: GET https://thekanaa.com/ar-sa/gaming-consoles.html?_rsc=pm4ao -&gt; net::ERR_ABORTED</t>
+  </si>
+  <si>
+    <t>Error: GET https://thekanaa.com/ar-sa/gaming-consoles.html?_rsc=pm4ao -&gt; net::ERR_ABORTED GET https://thekanaa.com/ar-sa/mobile-phones-tablets.html?_rsc=pm4ao -&gt; net::ERR_ABORTED [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m [32m- Expected - 1[39m [31m+ Received + 4[39m [32m- Array [][39m [31m+ Array [[39m [31m+ "GET https://thekanaa.com/ar-sa/gaming-consoles.html?_rsc=pm4ao -&gt; net::ERR_ABORTED",[39m [31m+ "GET https://thek</t>
+  </si>
+  <si>
+    <t>9161</t>
   </si>
   <si>
     <t>C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-065-2bb36-k-health-—-first-party-only-chromium\test-failed-1.png; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-065-2bb36-k-health-—-first-party-only-chromium\video.webm; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-065-2bb36-k-health-—-first-party-only-chromium\error-context.md; C:\Users\ThinkPad T480s Pro\Documents\homepage-ts-port\test-results\homepage-ui-TC-HOME-AR-065-2bb36-k-health-—-first-party-only-chromium\trace.zip</t>
@@ -647,19 +752,25 @@
     <t>TC-HOME-AR-005</t>
   </si>
   <si>
+    <t>تسوّّق حسب الماركة — inputs</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-005: تسوّّق حسب الماركة — input edge values</t>
   </si>
   <si>
-    <t>5687</t>
+    <t>7335</t>
   </si>
   <si>
     <t>TC-HOME-AR-052</t>
   </si>
   <si>
+    <t>تسوق حسب الفئة — inputs</t>
+  </si>
+  <si>
     <t>TC-HOME-AR-052: تسوق حسب الفئة — input edge values</t>
   </si>
   <si>
-    <t>1703</t>
+    <t>1982</t>
   </si>
   <si>
     <t>Change</t>
@@ -671,16 +782,64 @@
     <t>Detail</t>
   </si>
   <si>
+    <t>Added</t>
+  </si>
+  <si>
+    <t>ارتق إلى آيفون 18</t>
+  </si>
+  <si>
+    <t>New on the homepage since the previous scan; needs test coverage</t>
+  </si>
+  <si>
+    <t>جوالك الجديد وكل اللي تحتاجه معه.</t>
+  </si>
+  <si>
+    <t>سماعات ألعاب</t>
+  </si>
+  <si>
+    <t>Removed</t>
+  </si>
+  <si>
+    <t>تابلتك الجديد مع كل اللي تحتاجه.</t>
+  </si>
+  <si>
+    <t>Missing from the homepage; confirm the removal was intentional before changing the inventory</t>
+  </si>
+  <si>
+    <t>اشتر 1 واحصل على 1 مجانا</t>
+  </si>
+  <si>
+    <t>PS5 تسوق باقات</t>
+  </si>
+  <si>
+    <t>Changed</t>
+  </si>
+  <si>
+    <t>تسوّّق حسب الماركة</t>
+  </si>
+  <si>
+    <t>element counts {"buttons":26,"links":63,"inputs":2,"images":71,"sliders":1,"productCards":0} -&gt; {"buttons":26,"links":62,"inputs":2,"images":70,"sliders":1,"productCards":0}</t>
+  </si>
+  <si>
+    <t>اختاروا عطراً يستحق أن يكون هدية.</t>
+  </si>
+  <si>
+    <t>element counts {"buttons":16,"links":9,"inputs":0,"images":32,"sliders":0,"productCards":8} -&gt; {"buttons":16,"links":10,"inputs":0,"images":33,"sliders":0,"productCards":8}</t>
+  </si>
+  <si>
+    <t>منتجات مناسبة لكل عمر</t>
+  </si>
+  <si>
+    <t>element counts {"buttons":14,"links":14,"inputs":0,"images":35,"sliders":0,"productCards":7} -&gt; {"buttons":16,"links":15,"inputs":0,"images":39,"sliders":0,"productCards":8}</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Feature / section</t>
+  </si>
+  <si>
     <t>n/a</t>
-  </si>
-  <si>
-    <t>No discovery diff for this locale</t>
-  </si>
-  <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>Feature / section</t>
   </si>
   <si>
     <t>No plan changes recorded for this locale</t>
@@ -1126,7 +1285,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1134,7 +1293,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1305,10 +1464,10 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -1326,7 +1485,7 @@
         <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J3" t="s">
         <v>33</v>
@@ -1335,7 +1494,7 @@
         <v>15</v>
       </c>
       <c r="L3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M3" t="s">
         <v>15</v>
@@ -1346,13 +1505,13 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -1370,7 +1529,7 @@
         <v>15</v>
       </c>
       <c r="I4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J4" t="s">
         <v>33</v>
@@ -1379,7 +1538,7 @@
         <v>15</v>
       </c>
       <c r="L4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="M4" t="s">
         <v>15</v>
@@ -1390,13 +1549,13 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
@@ -1414,7 +1573,7 @@
         <v>15</v>
       </c>
       <c r="I5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J5" t="s">
         <v>33</v>
@@ -1423,7 +1582,7 @@
         <v>15</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="M5" t="s">
         <v>15</v>
@@ -1434,13 +1593,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -1458,7 +1617,7 @@
         <v>15</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J6" t="s">
         <v>33</v>
@@ -1467,7 +1626,7 @@
         <v>15</v>
       </c>
       <c r="L6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="M6" t="s">
         <v>15</v>
@@ -1478,13 +1637,13 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
@@ -1502,7 +1661,7 @@
         <v>15</v>
       </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J7" t="s">
         <v>33</v>
@@ -1511,7 +1670,7 @@
         <v>15</v>
       </c>
       <c r="L7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="M7" t="s">
         <v>15</v>
@@ -1522,13 +1681,13 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -1546,7 +1705,7 @@
         <v>15</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="J8" t="s">
         <v>33</v>
@@ -1555,7 +1714,7 @@
         <v>15</v>
       </c>
       <c r="L8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="M8" t="s">
         <v>15</v>
@@ -1566,13 +1725,13 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
@@ -1590,7 +1749,7 @@
         <v>15</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="J9" t="s">
         <v>33</v>
@@ -1599,7 +1758,7 @@
         <v>15</v>
       </c>
       <c r="L9" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="M9" t="s">
         <v>15</v>
@@ -1610,13 +1769,13 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -1634,7 +1793,7 @@
         <v>15</v>
       </c>
       <c r="I10" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="J10" t="s">
         <v>33</v>
@@ -1643,7 +1802,7 @@
         <v>15</v>
       </c>
       <c r="L10" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="M10" t="s">
         <v>15</v>
@@ -1654,13 +1813,13 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1678,7 +1837,7 @@
         <v>15</v>
       </c>
       <c r="I11" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
         <v>33</v>
@@ -1687,7 +1846,7 @@
         <v>15</v>
       </c>
       <c r="L11" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="M11" t="s">
         <v>15</v>
@@ -1698,13 +1857,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
@@ -1722,7 +1881,7 @@
         <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s">
         <v>33</v>
@@ -1731,7 +1890,7 @@
         <v>15</v>
       </c>
       <c r="L12" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="M12" t="s">
         <v>15</v>
@@ -1742,13 +1901,13 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -1766,7 +1925,7 @@
         <v>15</v>
       </c>
       <c r="I13" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="J13" t="s">
         <v>33</v>
@@ -1775,7 +1934,7 @@
         <v>15</v>
       </c>
       <c r="L13" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="M13" t="s">
         <v>15</v>
@@ -1786,13 +1945,13 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1810,7 +1969,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="J14" t="s">
         <v>33</v>
@@ -1819,7 +1978,7 @@
         <v>15</v>
       </c>
       <c r="L14" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="M14" t="s">
         <v>15</v>
@@ -1830,13 +1989,13 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1847,26 +2006,26 @@
       <c r="F15" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>8</v>
+      <c r="G15" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H15" t="s">
         <v>15</v>
       </c>
       <c r="I15" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="J15" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="K15" t="s">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="L15" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="M15" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="N15" t="s">
         <v>15</v>
@@ -1874,13 +2033,13 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -1891,23 +2050,23 @@
       <c r="F16" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>8</v>
+      <c r="G16" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
       </c>
       <c r="I16" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="J16" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K16" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L16" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="M16" t="s">
         <v>15</v>
@@ -1918,13 +2077,13 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -1935,23 +2094,23 @@
       <c r="F17" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>8</v>
+      <c r="G17" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
       </c>
       <c r="I17" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="J17" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K17" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L17" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="M17" t="s">
         <v>15</v>
@@ -1962,13 +2121,13 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1979,23 +2138,23 @@
       <c r="F18" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>8</v>
+      <c r="G18" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H18" t="s">
         <v>15</v>
       </c>
       <c r="I18" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="J18" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K18" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L18" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="M18" t="s">
         <v>15</v>
@@ -2006,13 +2165,13 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
@@ -2023,23 +2182,23 @@
       <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>8</v>
+      <c r="G19" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H19" t="s">
         <v>15</v>
       </c>
       <c r="I19" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="J19" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K19" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L19" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="M19" t="s">
         <v>15</v>
@@ -2050,13 +2209,13 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -2074,7 +2233,7 @@
         <v>15</v>
       </c>
       <c r="I20" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="J20" t="s">
         <v>33</v>
@@ -2083,7 +2242,7 @@
         <v>15</v>
       </c>
       <c r="L20" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="M20" t="s">
         <v>15</v>
@@ -2094,13 +2253,13 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -2118,7 +2277,7 @@
         <v>15</v>
       </c>
       <c r="I21" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="J21" t="s">
         <v>33</v>
@@ -2127,7 +2286,7 @@
         <v>15</v>
       </c>
       <c r="L21" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="M21" t="s">
         <v>15</v>
@@ -2138,13 +2297,13 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>111</v>
       </c>
       <c r="C22" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -2162,7 +2321,7 @@
         <v>15</v>
       </c>
       <c r="I22" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="J22" t="s">
         <v>33</v>
@@ -2171,7 +2330,7 @@
         <v>15</v>
       </c>
       <c r="L22" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="M22" t="s">
         <v>15</v>
@@ -2182,13 +2341,13 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>115</v>
       </c>
       <c r="C23" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -2206,7 +2365,7 @@
         <v>15</v>
       </c>
       <c r="I23" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="J23" t="s">
         <v>33</v>
@@ -2215,7 +2374,7 @@
         <v>15</v>
       </c>
       <c r="L23" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="M23" t="s">
         <v>15</v>
@@ -2226,13 +2385,13 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D24" t="s">
         <v>5</v>
@@ -2250,7 +2409,7 @@
         <v>15</v>
       </c>
       <c r="I24" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="J24" t="s">
         <v>33</v>
@@ -2259,7 +2418,7 @@
         <v>15</v>
       </c>
       <c r="L24" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="M24" t="s">
         <v>15</v>
@@ -2270,13 +2429,13 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="D25" t="s">
         <v>5</v>
@@ -2294,7 +2453,7 @@
         <v>15</v>
       </c>
       <c r="I25" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="J25" t="s">
         <v>33</v>
@@ -2303,7 +2462,7 @@
         <v>15</v>
       </c>
       <c r="L25" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="M25" t="s">
         <v>15</v>
@@ -2314,13 +2473,13 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
         <v>5</v>
@@ -2338,7 +2497,7 @@
         <v>15</v>
       </c>
       <c r="I26" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="J26" t="s">
         <v>33</v>
@@ -2347,7 +2506,7 @@
         <v>15</v>
       </c>
       <c r="L26" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="M26" t="s">
         <v>15</v>
@@ -2358,13 +2517,13 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
         <v>5</v>
@@ -2382,7 +2541,7 @@
         <v>15</v>
       </c>
       <c r="I27" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="J27" t="s">
         <v>33</v>
@@ -2391,7 +2550,7 @@
         <v>15</v>
       </c>
       <c r="L27" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="M27" t="s">
         <v>15</v>
@@ -2402,13 +2561,13 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C28" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="D28" t="s">
         <v>5</v>
@@ -2426,19 +2585,19 @@
         <v>15</v>
       </c>
       <c r="I28" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="J28" t="s">
-        <v>74</v>
+        <v>137</v>
       </c>
       <c r="K28" t="s">
-        <v>74</v>
+        <v>137</v>
       </c>
       <c r="L28" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="M28" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="N28" t="s">
         <v>15</v>
@@ -2446,13 +2605,13 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="B29" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="C29" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="D29" t="s">
         <v>5</v>
@@ -2463,26 +2622,26 @@
       <c r="F29" t="s">
         <v>16</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>7</v>
+      <c r="G29" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="H29" t="s">
         <v>15</v>
       </c>
       <c r="I29" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="J29" t="s">
-        <v>33</v>
+        <v>143</v>
       </c>
       <c r="K29" t="s">
-        <v>15</v>
+        <v>144</v>
       </c>
       <c r="L29" t="s">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="M29" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="N29" t="s">
         <v>15</v>
@@ -2490,13 +2649,13 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>148</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="D30" t="s">
         <v>5</v>
@@ -2514,7 +2673,7 @@
         <v>15</v>
       </c>
       <c r="I30" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="J30" t="s">
         <v>33</v>
@@ -2523,7 +2682,7 @@
         <v>15</v>
       </c>
       <c r="L30" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="M30" t="s">
         <v>15</v>
@@ -2534,13 +2693,13 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>122</v>
+        <v>151</v>
       </c>
       <c r="B31" t="s">
-        <v>123</v>
+        <v>152</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>153</v>
       </c>
       <c r="D31" t="s">
         <v>5</v>
@@ -2558,19 +2717,19 @@
         <v>15</v>
       </c>
       <c r="I31" t="s">
-        <v>124</v>
+        <v>153</v>
       </c>
       <c r="J31" t="s">
-        <v>79</v>
+        <v>154</v>
       </c>
       <c r="K31" t="s">
-        <v>79</v>
+        <v>155</v>
       </c>
       <c r="L31" t="s">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="M31" t="s">
-        <v>15</v>
+        <v>157</v>
       </c>
       <c r="N31" t="s">
         <v>15</v>
@@ -2578,13 +2737,13 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>159</v>
       </c>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="D32" t="s">
         <v>5</v>
@@ -2595,23 +2754,23 @@
       <c r="F32" t="s">
         <v>16</v>
       </c>
-      <c r="G32" s="3" t="s">
-        <v>8</v>
+      <c r="G32" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H32" t="s">
         <v>15</v>
       </c>
       <c r="I32" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="J32" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K32" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L32" t="s">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="M32" t="s">
         <v>15</v>
@@ -2622,13 +2781,13 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
       <c r="D33" t="s">
         <v>5</v>
@@ -2639,23 +2798,23 @@
       <c r="F33" t="s">
         <v>16</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>8</v>
+      <c r="G33" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H33" t="s">
         <v>15</v>
       </c>
       <c r="I33" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
       <c r="J33" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K33" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L33" t="s">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="M33" t="s">
         <v>15</v>
@@ -2666,13 +2825,13 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>129</v>
+        <v>166</v>
       </c>
       <c r="B34" t="s">
-        <v>123</v>
+        <v>167</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="D34" t="s">
         <v>5</v>
@@ -2683,23 +2842,23 @@
       <c r="F34" t="s">
         <v>16</v>
       </c>
-      <c r="G34" s="3" t="s">
-        <v>8</v>
+      <c r="G34" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H34" t="s">
         <v>15</v>
       </c>
       <c r="I34" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="J34" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="K34" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="L34" t="s">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="M34" t="s">
         <v>15</v>
@@ -2710,13 +2869,13 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="B35" t="s">
-        <v>123</v>
+        <v>171</v>
       </c>
       <c r="C35" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="D35" t="s">
         <v>5</v>
@@ -2734,7 +2893,7 @@
         <v>15</v>
       </c>
       <c r="I35" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="J35" t="s">
         <v>33</v>
@@ -2743,7 +2902,7 @@
         <v>15</v>
       </c>
       <c r="L35" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="M35" t="s">
         <v>15</v>
@@ -2754,13 +2913,13 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
       <c r="B36" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>176</v>
       </c>
       <c r="D36" t="s">
         <v>5</v>
@@ -2778,7 +2937,7 @@
         <v>15</v>
       </c>
       <c r="I36" t="s">
-        <v>135</v>
+        <v>176</v>
       </c>
       <c r="J36" t="s">
         <v>33</v>
@@ -2787,7 +2946,7 @@
         <v>15</v>
       </c>
       <c r="L36" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="M36" t="s">
         <v>15</v>
@@ -2798,13 +2957,13 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>137</v>
+        <v>178</v>
       </c>
       <c r="B37" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
       <c r="C37" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="D37" t="s">
         <v>5</v>
@@ -2822,7 +2981,7 @@
         <v>15</v>
       </c>
       <c r="I37" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="J37" t="s">
         <v>33</v>
@@ -2831,7 +2990,7 @@
         <v>15</v>
       </c>
       <c r="L37" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="M37" t="s">
         <v>15</v>
@@ -2842,13 +3001,13 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="B38" t="s">
-        <v>123</v>
+        <v>183</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>184</v>
       </c>
       <c r="D38" t="s">
         <v>5</v>
@@ -2866,7 +3025,7 @@
         <v>15</v>
       </c>
       <c r="I38" t="s">
-        <v>141</v>
+        <v>184</v>
       </c>
       <c r="J38" t="s">
         <v>33</v>
@@ -2875,7 +3034,7 @@
         <v>15</v>
       </c>
       <c r="L38" t="s">
-        <v>142</v>
+        <v>185</v>
       </c>
       <c r="M38" t="s">
         <v>15</v>
@@ -2886,13 +3045,13 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>143</v>
+        <v>186</v>
       </c>
       <c r="B39" t="s">
-        <v>123</v>
+        <v>187</v>
       </c>
       <c r="C39" t="s">
-        <v>144</v>
+        <v>188</v>
       </c>
       <c r="D39" t="s">
         <v>5</v>
@@ -2910,7 +3069,7 @@
         <v>15</v>
       </c>
       <c r="I39" t="s">
-        <v>144</v>
+        <v>188</v>
       </c>
       <c r="J39" t="s">
         <v>33</v>
@@ -2919,7 +3078,7 @@
         <v>15</v>
       </c>
       <c r="L39" t="s">
-        <v>145</v>
+        <v>189</v>
       </c>
       <c r="M39" t="s">
         <v>15</v>
@@ -2930,13 +3089,13 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="B40" t="s">
-        <v>147</v>
+        <v>191</v>
       </c>
       <c r="C40" t="s">
-        <v>148</v>
+        <v>192</v>
       </c>
       <c r="D40" t="s">
         <v>5</v>
@@ -2954,7 +3113,7 @@
         <v>15</v>
       </c>
       <c r="I40" t="s">
-        <v>148</v>
+        <v>192</v>
       </c>
       <c r="J40" t="s">
         <v>33</v>
@@ -2963,7 +3122,7 @@
         <v>15</v>
       </c>
       <c r="L40" t="s">
-        <v>149</v>
+        <v>193</v>
       </c>
       <c r="M40" t="s">
         <v>15</v>
@@ -2974,13 +3133,13 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>150</v>
+        <v>194</v>
       </c>
       <c r="B41" t="s">
-        <v>147</v>
+        <v>195</v>
       </c>
       <c r="C41" t="s">
-        <v>151</v>
+        <v>196</v>
       </c>
       <c r="D41" t="s">
         <v>5</v>
@@ -2998,7 +3157,7 @@
         <v>15</v>
       </c>
       <c r="I41" t="s">
-        <v>151</v>
+        <v>196</v>
       </c>
       <c r="J41" t="s">
         <v>33</v>
@@ -3007,7 +3166,7 @@
         <v>15</v>
       </c>
       <c r="L41" t="s">
-        <v>152</v>
+        <v>197</v>
       </c>
       <c r="M41" t="s">
         <v>15</v>
@@ -3018,13 +3177,13 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>153</v>
+        <v>198</v>
       </c>
       <c r="B42" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="C42" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
@@ -3035,26 +3194,26 @@
       <c r="F42" t="s">
         <v>16</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>8</v>
+      <c r="G42" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H42" t="s">
         <v>15</v>
       </c>
       <c r="I42" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="J42" t="s">
-        <v>155</v>
+        <v>33</v>
       </c>
       <c r="K42" t="s">
-        <v>156</v>
+        <v>15</v>
       </c>
       <c r="L42" t="s">
-        <v>157</v>
+        <v>201</v>
       </c>
       <c r="M42" t="s">
-        <v>158</v>
+        <v>15</v>
       </c>
       <c r="N42" t="s">
         <v>15</v>
@@ -3062,13 +3221,13 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>159</v>
+        <v>202</v>
       </c>
       <c r="B43" t="s">
-        <v>147</v>
+        <v>203</v>
       </c>
       <c r="C43" t="s">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="D43" t="s">
         <v>5</v>
@@ -3079,26 +3238,26 @@
       <c r="F43" t="s">
         <v>16</v>
       </c>
-      <c r="G43" s="3" t="s">
-        <v>8</v>
+      <c r="G43" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H43" t="s">
         <v>15</v>
       </c>
       <c r="I43" t="s">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="J43" t="s">
-        <v>161</v>
+        <v>33</v>
       </c>
       <c r="K43" t="s">
-        <v>162</v>
+        <v>15</v>
       </c>
       <c r="L43" t="s">
-        <v>163</v>
+        <v>205</v>
       </c>
       <c r="M43" t="s">
-        <v>164</v>
+        <v>15</v>
       </c>
       <c r="N43" t="s">
         <v>15</v>
@@ -3106,13 +3265,13 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>165</v>
+        <v>206</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>207</v>
       </c>
       <c r="C44" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="D44" t="s">
         <v>5</v>
@@ -3123,26 +3282,26 @@
       <c r="F44" t="s">
         <v>16</v>
       </c>
-      <c r="G44" s="3" t="s">
-        <v>8</v>
+      <c r="G44" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H44" t="s">
         <v>15</v>
       </c>
       <c r="I44" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="J44" t="s">
-        <v>167</v>
+        <v>33</v>
       </c>
       <c r="K44" t="s">
-        <v>168</v>
+        <v>15</v>
       </c>
       <c r="L44" t="s">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="M44" t="s">
-        <v>170</v>
+        <v>15</v>
       </c>
       <c r="N44" t="s">
         <v>15</v>
@@ -3150,13 +3309,13 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>171</v>
+        <v>210</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>211</v>
       </c>
       <c r="C45" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
@@ -3167,26 +3326,26 @@
       <c r="F45" t="s">
         <v>16</v>
       </c>
-      <c r="G45" s="3" t="s">
-        <v>8</v>
+      <c r="G45" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H45" t="s">
         <v>15</v>
       </c>
       <c r="I45" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="J45" t="s">
-        <v>173</v>
+        <v>33</v>
       </c>
       <c r="K45" t="s">
-        <v>174</v>
+        <v>15</v>
       </c>
       <c r="L45" t="s">
-        <v>175</v>
+        <v>213</v>
       </c>
       <c r="M45" t="s">
-        <v>176</v>
+        <v>15</v>
       </c>
       <c r="N45" t="s">
         <v>15</v>
@@ -3194,13 +3353,13 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>177</v>
+        <v>214</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>215</v>
       </c>
       <c r="C46" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
       <c r="D46" t="s">
         <v>5</v>
@@ -3211,26 +3370,26 @@
       <c r="F46" t="s">
         <v>16</v>
       </c>
-      <c r="G46" s="3" t="s">
-        <v>8</v>
+      <c r="G46" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H46" t="s">
         <v>15</v>
       </c>
       <c r="I46" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
       <c r="J46" t="s">
-        <v>179</v>
+        <v>33</v>
       </c>
       <c r="K46" t="s">
-        <v>180</v>
+        <v>15</v>
       </c>
       <c r="L46" t="s">
-        <v>181</v>
+        <v>217</v>
       </c>
       <c r="M46" t="s">
-        <v>182</v>
+        <v>15</v>
       </c>
       <c r="N46" t="s">
         <v>15</v>
@@ -3238,13 +3397,13 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>183</v>
+        <v>218</v>
       </c>
       <c r="B47" t="s">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="C47" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="D47" t="s">
         <v>5</v>
@@ -3262,19 +3421,19 @@
         <v>15</v>
       </c>
       <c r="I47" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="J47" t="s">
-        <v>186</v>
+        <v>221</v>
       </c>
       <c r="K47" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
       <c r="L47" t="s">
-        <v>188</v>
+        <v>223</v>
       </c>
       <c r="M47" t="s">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="N47" t="s">
         <v>15</v>
@@ -3282,13 +3441,13 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>190</v>
+        <v>225</v>
       </c>
       <c r="B48" t="s">
-        <v>191</v>
+        <v>226</v>
       </c>
       <c r="C48" t="s">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="D48" t="s">
         <v>5</v>
@@ -3306,7 +3465,7 @@
         <v>15</v>
       </c>
       <c r="I48" t="s">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="J48" t="s">
         <v>33</v>
@@ -3315,7 +3474,7 @@
         <v>15</v>
       </c>
       <c r="L48" t="s">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="M48" t="s">
         <v>15</v>
@@ -3326,13 +3485,13 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="B49" t="s">
-        <v>191</v>
+        <v>230</v>
       </c>
       <c r="C49" t="s">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="D49" t="s">
         <v>5</v>
@@ -3350,7 +3509,7 @@
         <v>15</v>
       </c>
       <c r="I49" t="s">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="J49" t="s">
         <v>33</v>
@@ -3359,7 +3518,7 @@
         <v>15</v>
       </c>
       <c r="L49" t="s">
-        <v>196</v>
+        <v>232</v>
       </c>
       <c r="M49" t="s">
         <v>15</v>
@@ -3370,13 +3529,13 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>197</v>
+        <v>233</v>
       </c>
       <c r="B50" t="s">
-        <v>191</v>
+        <v>234</v>
       </c>
       <c r="C50" t="s">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="D50" t="s">
         <v>5</v>
@@ -3387,26 +3546,26 @@
       <c r="F50" t="s">
         <v>16</v>
       </c>
-      <c r="G50" s="3" t="s">
-        <v>8</v>
+      <c r="G50" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="H50" t="s">
         <v>15</v>
       </c>
       <c r="I50" t="s">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="J50" t="s">
-        <v>199</v>
+        <v>33</v>
       </c>
       <c r="K50" t="s">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="L50" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="M50" t="s">
-        <v>202</v>
+        <v>15</v>
       </c>
       <c r="N50" t="s">
         <v>15</v>
@@ -3414,13 +3573,13 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>203</v>
+        <v>237</v>
       </c>
       <c r="B51" t="s">
-        <v>191</v>
+        <v>238</v>
       </c>
       <c r="C51" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="D51" t="s">
         <v>5</v>
@@ -3438,19 +3597,19 @@
         <v>15</v>
       </c>
       <c r="I51" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="J51" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="K51" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="L51" t="s">
-        <v>207</v>
+        <v>242</v>
       </c>
       <c r="M51" t="s">
-        <v>208</v>
+        <v>243</v>
       </c>
       <c r="N51" t="s">
         <v>15</v>
@@ -3458,13 +3617,13 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>209</v>
+        <v>244</v>
       </c>
       <c r="B52" t="s">
-        <v>191</v>
+        <v>245</v>
       </c>
       <c r="C52" t="s">
-        <v>210</v>
+        <v>246</v>
       </c>
       <c r="D52" t="s">
         <v>5</v>
@@ -3482,7 +3641,7 @@
         <v>15</v>
       </c>
       <c r="I52" t="s">
-        <v>210</v>
+        <v>246</v>
       </c>
       <c r="J52" t="s">
         <v>33</v>
@@ -3491,7 +3650,7 @@
         <v>15</v>
       </c>
       <c r="L52" t="s">
-        <v>211</v>
+        <v>247</v>
       </c>
       <c r="M52" t="s">
         <v>15</v>
@@ -3502,13 +3661,13 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="B53" t="s">
-        <v>191</v>
+        <v>249</v>
       </c>
       <c r="C53" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="D53" t="s">
         <v>5</v>
@@ -3526,7 +3685,7 @@
         <v>15</v>
       </c>
       <c r="I53" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="J53" t="s">
         <v>33</v>
@@ -3535,7 +3694,7 @@
         <v>15</v>
       </c>
       <c r="L53" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="M53" t="s">
         <v>15</v>
@@ -3553,7 +3712,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -3618,13 +3777,13 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>134</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>136</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -3642,19 +3801,19 @@
         <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>73</v>
+        <v>136</v>
       </c>
       <c r="J2" t="s">
-        <v>74</v>
+        <v>137</v>
       </c>
       <c r="K2" t="s">
-        <v>74</v>
+        <v>137</v>
       </c>
       <c r="L2" t="s">
-        <v>75</v>
+        <v>138</v>
       </c>
       <c r="M2" t="s">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="N2" t="s">
         <v>15</v>
@@ -3662,13 +3821,13 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>140</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>142</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -3686,19 +3845,19 @@
         <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>78</v>
+        <v>142</v>
       </c>
       <c r="J3" t="s">
-        <v>79</v>
+        <v>143</v>
       </c>
       <c r="K3" t="s">
-        <v>79</v>
+        <v>144</v>
       </c>
       <c r="L3" t="s">
-        <v>80</v>
+        <v>145</v>
       </c>
       <c r="M3" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="N3" t="s">
         <v>15</v>
@@ -3706,13 +3865,13 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>153</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -3730,19 +3889,19 @@
         <v>15</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>153</v>
       </c>
       <c r="J4" t="s">
-        <v>79</v>
+        <v>154</v>
       </c>
       <c r="K4" t="s">
-        <v>79</v>
+        <v>155</v>
       </c>
       <c r="L4" t="s">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="M4" t="s">
-        <v>15</v>
+        <v>157</v>
       </c>
       <c r="N4" t="s">
         <v>15</v>
@@ -3750,13 +3909,13 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>218</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>219</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>220</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
@@ -3774,19 +3933,19 @@
         <v>15</v>
       </c>
       <c r="I5" t="s">
-        <v>84</v>
+        <v>220</v>
       </c>
       <c r="J5" t="s">
-        <v>79</v>
+        <v>221</v>
       </c>
       <c r="K5" t="s">
-        <v>79</v>
+        <v>222</v>
       </c>
       <c r="L5" t="s">
-        <v>80</v>
+        <v>223</v>
       </c>
       <c r="M5" t="s">
-        <v>15</v>
+        <v>224</v>
       </c>
       <c r="N5" t="s">
         <v>15</v>
@@ -3794,13 +3953,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>237</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>238</v>
       </c>
       <c r="C6" t="s">
-        <v>86</v>
+        <v>239</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -3818,593 +3977,21 @@
         <v>15</v>
       </c>
       <c r="I6" t="s">
-        <v>86</v>
+        <v>239</v>
       </c>
       <c r="J6" t="s">
-        <v>79</v>
+        <v>240</v>
       </c>
       <c r="K6" t="s">
-        <v>79</v>
+        <v>241</v>
       </c>
       <c r="L6" t="s">
-        <v>80</v>
+        <v>242</v>
       </c>
       <c r="M6" t="s">
-        <v>15</v>
+        <v>243</v>
       </c>
       <c r="N6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" t="s">
-        <v>112</v>
-      </c>
-      <c r="D7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>112</v>
-      </c>
-      <c r="J7" t="s">
-        <v>74</v>
-      </c>
-      <c r="K7" t="s">
-        <v>74</v>
-      </c>
-      <c r="L7" t="s">
-        <v>113</v>
-      </c>
-      <c r="M7" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>122</v>
-      </c>
-      <c r="B8" t="s">
-        <v>123</v>
-      </c>
-      <c r="C8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D8" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" t="s">
-        <v>124</v>
-      </c>
-      <c r="J8" t="s">
-        <v>79</v>
-      </c>
-      <c r="K8" t="s">
-        <v>79</v>
-      </c>
-      <c r="L8" t="s">
-        <v>80</v>
-      </c>
-      <c r="M8" t="s">
-        <v>15</v>
-      </c>
-      <c r="N8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>125</v>
-      </c>
-      <c r="B9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D9" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" t="s">
-        <v>126</v>
-      </c>
-      <c r="J9" t="s">
-        <v>79</v>
-      </c>
-      <c r="K9" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9" t="s">
-        <v>80</v>
-      </c>
-      <c r="M9" t="s">
-        <v>15</v>
-      </c>
-      <c r="N9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" t="s">
-        <v>123</v>
-      </c>
-      <c r="C10" t="s">
-        <v>128</v>
-      </c>
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H10" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" t="s">
-        <v>128</v>
-      </c>
-      <c r="J10" t="s">
-        <v>79</v>
-      </c>
-      <c r="K10" t="s">
-        <v>79</v>
-      </c>
-      <c r="L10" t="s">
-        <v>80</v>
-      </c>
-      <c r="M10" t="s">
-        <v>15</v>
-      </c>
-      <c r="N10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>129</v>
-      </c>
-      <c r="B11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C11" t="s">
-        <v>130</v>
-      </c>
-      <c r="D11" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" t="s">
-        <v>3</v>
-      </c>
-      <c r="F11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" t="s">
-        <v>130</v>
-      </c>
-      <c r="J11" t="s">
-        <v>79</v>
-      </c>
-      <c r="K11" t="s">
-        <v>79</v>
-      </c>
-      <c r="L11" t="s">
-        <v>80</v>
-      </c>
-      <c r="M11" t="s">
-        <v>15</v>
-      </c>
-      <c r="N11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" t="s">
-        <v>147</v>
-      </c>
-      <c r="C12" t="s">
-        <v>154</v>
-      </c>
-      <c r="D12" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" t="s">
-        <v>154</v>
-      </c>
-      <c r="J12" t="s">
-        <v>155</v>
-      </c>
-      <c r="K12" t="s">
-        <v>156</v>
-      </c>
-      <c r="L12" t="s">
-        <v>157</v>
-      </c>
-      <c r="M12" t="s">
-        <v>158</v>
-      </c>
-      <c r="N12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>159</v>
-      </c>
-      <c r="B13" t="s">
-        <v>147</v>
-      </c>
-      <c r="C13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D13" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" t="s">
-        <v>160</v>
-      </c>
-      <c r="J13" t="s">
-        <v>161</v>
-      </c>
-      <c r="K13" t="s">
-        <v>162</v>
-      </c>
-      <c r="L13" t="s">
-        <v>163</v>
-      </c>
-      <c r="M13" t="s">
-        <v>164</v>
-      </c>
-      <c r="N13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" t="s">
-        <v>147</v>
-      </c>
-      <c r="C14" t="s">
-        <v>166</v>
-      </c>
-      <c r="D14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" t="s">
-        <v>166</v>
-      </c>
-      <c r="J14" t="s">
-        <v>167</v>
-      </c>
-      <c r="K14" t="s">
-        <v>168</v>
-      </c>
-      <c r="L14" t="s">
-        <v>169</v>
-      </c>
-      <c r="M14" t="s">
-        <v>170</v>
-      </c>
-      <c r="N14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>171</v>
-      </c>
-      <c r="B15" t="s">
-        <v>147</v>
-      </c>
-      <c r="C15" t="s">
-        <v>172</v>
-      </c>
-      <c r="D15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" t="s">
-        <v>172</v>
-      </c>
-      <c r="J15" t="s">
-        <v>173</v>
-      </c>
-      <c r="K15" t="s">
-        <v>174</v>
-      </c>
-      <c r="L15" t="s">
-        <v>175</v>
-      </c>
-      <c r="M15" t="s">
-        <v>176</v>
-      </c>
-      <c r="N15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>177</v>
-      </c>
-      <c r="B16" t="s">
-        <v>147</v>
-      </c>
-      <c r="C16" t="s">
-        <v>178</v>
-      </c>
-      <c r="D16" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H16" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" t="s">
-        <v>178</v>
-      </c>
-      <c r="J16" t="s">
-        <v>179</v>
-      </c>
-      <c r="K16" t="s">
-        <v>180</v>
-      </c>
-      <c r="L16" t="s">
-        <v>181</v>
-      </c>
-      <c r="M16" t="s">
-        <v>182</v>
-      </c>
-      <c r="N16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>183</v>
-      </c>
-      <c r="B17" t="s">
-        <v>184</v>
-      </c>
-      <c r="C17" t="s">
-        <v>185</v>
-      </c>
-      <c r="D17" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" t="s">
-        <v>185</v>
-      </c>
-      <c r="J17" t="s">
-        <v>186</v>
-      </c>
-      <c r="K17" t="s">
-        <v>187</v>
-      </c>
-      <c r="L17" t="s">
-        <v>188</v>
-      </c>
-      <c r="M17" t="s">
-        <v>189</v>
-      </c>
-      <c r="N17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>197</v>
-      </c>
-      <c r="B18" t="s">
-        <v>191</v>
-      </c>
-      <c r="C18" t="s">
-        <v>198</v>
-      </c>
-      <c r="D18" t="s">
-        <v>5</v>
-      </c>
-      <c r="E18" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I18" t="s">
-        <v>198</v>
-      </c>
-      <c r="J18" t="s">
-        <v>199</v>
-      </c>
-      <c r="K18" t="s">
-        <v>200</v>
-      </c>
-      <c r="L18" t="s">
-        <v>201</v>
-      </c>
-      <c r="M18" t="s">
-        <v>202</v>
-      </c>
-      <c r="N18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>203</v>
-      </c>
-      <c r="B19" t="s">
-        <v>191</v>
-      </c>
-      <c r="C19" t="s">
-        <v>204</v>
-      </c>
-      <c r="D19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E19" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H19" t="s">
-        <v>15</v>
-      </c>
-      <c r="I19" t="s">
-        <v>204</v>
-      </c>
-      <c r="J19" t="s">
-        <v>205</v>
-      </c>
-      <c r="K19" t="s">
-        <v>206</v>
-      </c>
-      <c r="L19" t="s">
-        <v>207</v>
-      </c>
-      <c r="M19" t="s">
-        <v>208</v>
-      </c>
-      <c r="N19" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4417,7 +4004,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -4427,24 +4014,112 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>256</v>
       </c>
       <c r="C2" t="s">
-        <v>219</v>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C8" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>265</v>
+      </c>
+      <c r="B9" t="s">
+        <v>268</v>
+      </c>
+      <c r="C9" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>265</v>
+      </c>
+      <c r="B10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C10" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4465,10 +4140,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>272</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>221</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>22</v>
@@ -4476,13 +4151,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>274</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>222</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>